<commit_message>
update files and bugs
</commit_message>
<xml_diff>
--- a/Data/Results Files Log.xlsx
+++ b/Data/Results Files Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Jack\OneDrive - SEI\Yolo_Website\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{467FD53A-4AF0-4233-9F8C-DF79DFC51549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A6F8C8-F5F9-49F0-90F7-82E872DB9FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{B2597F6E-531F-4750-96F4-BBEC03A736ED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B2597F6E-531F-4750-96F4-BBEC03A736ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="74">
   <si>
     <t>Groundwater Storage.csv</t>
   </si>
@@ -213,9 +213,6 @@
   </si>
   <si>
     <t>historical avg</t>
-  </si>
-  <si>
-    <t>user must update annually</t>
   </si>
   <si>
     <t>Reservoir Release-Capay Dam.csv</t>
@@ -667,14 +664,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B3E5313-6531-476C-969E-E5EB0B39DD2B}">
   <dimension ref="A1:G52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="53.6640625" customWidth="1"/>
-    <col min="2" max="3" width="18.109375" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" customWidth="1"/>
+    <col min="1" max="1" width="53.7109375" customWidth="1"/>
+    <col min="2" max="3" width="18.140625" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -682,7 +679,7 @@
         <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>49</v>
@@ -691,7 +688,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -702,10 +699,10 @@
         <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -716,10 +713,10 @@
         <v>46</v>
       </c>
       <c r="G3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -730,10 +727,10 @@
         <v>42</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -744,10 +741,10 @@
         <v>45</v>
       </c>
       <c r="G5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -761,10 +758,10 @@
         <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -775,7 +772,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -786,7 +783,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -797,7 +794,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -808,7 +805,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -819,7 +816,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -830,7 +827,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -841,7 +838,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -852,7 +849,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -863,7 +860,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -874,7 +871,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -885,7 +882,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>39</v>
       </c>
@@ -896,10 +893,10 @@
         <v>54</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>56</v>
       </c>
@@ -910,21 +907,21 @@
         <v>53</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -935,7 +932,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -946,7 +943,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -957,7 +954,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -968,9 +965,9 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
         <v>42</v>
@@ -979,7 +976,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -990,7 +987,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>22</v>
       </c>
@@ -1001,21 +998,21 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" t="s">
+        <v>42</v>
+      </c>
+      <c r="C28" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>60</v>
       </c>
-      <c r="B28" t="s">
-        <v>42</v>
-      </c>
-      <c r="C28" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>61</v>
-      </c>
       <c r="B29" t="s">
         <v>42</v>
       </c>
@@ -1023,7 +1020,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -1031,7 +1028,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -1039,7 +1036,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1047,10 +1044,10 @@
         <v>52</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -1058,7 +1055,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1069,7 +1066,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>15</v>
       </c>
@@ -1080,7 +1077,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>16</v>
       </c>
@@ -1091,7 +1088,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -1102,7 +1099,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>12</v>
       </c>
@@ -1113,7 +1110,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>13</v>
       </c>
@@ -1124,7 +1121,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>2</v>
       </c>
@@ -1135,7 +1132,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -1146,7 +1143,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1157,7 +1154,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>5</v>
       </c>
@@ -1168,7 +1165,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -1179,9 +1176,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>50</v>
@@ -1190,7 +1187,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>7</v>
       </c>
@@ -1201,7 +1198,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>8</v>
       </c>
@@ -1212,7 +1209,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>40</v>
       </c>
@@ -1223,7 +1220,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>14</v>
       </c>
@@ -1234,20 +1231,20 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B50" t="s">
         <v>52</v>
       </c>
       <c r="C50" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B51" t="s">
         <v>42</v>
@@ -1256,15 +1253,15 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B52" t="s">
         <v>52</v>
       </c>
       <c r="C52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>